<commit_message>
data : run pipeline complet Partage + La_French + Zen (sauvegarde)
Sauvegarde des fichiers finaux et intermediaires apres le run complet
avec tous les fixes (commits 62405ca, a1bf3ac, fee528f) :

- 3 fichiers Resultats/resultats_final_<P>.{csv,xlsx} :
  - Partage   : 43 lignes
  - La_French : 894 lignes
  - Zen       : 1184 lignes

- Pipeline/ : fichiers intermediaires (albums_a_rechercher,
  albums_match_complet, resultats_cotes) pour les 3 playlists.

- Bibliotheque/ : snapshot biblio scannee (11k+ albums).

- Playlists_Spotify/{Partage,Zen}.csv : mises a jour utilisateur.

Pas commite : debug_selection.csv (log technique 845K).
</commit_message>
<xml_diff>
--- a/data/Resultats/resultats_final_Partage.xlsx
+++ b/data/Resultats/resultats_final_Partage.xlsx
@@ -413,183 +413,187 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Sources Qobuz</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Sources Bibli</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Artist_A_rechercher</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Artist_Possede</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Artist_sim</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Album_A_rechercher</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Album_Possede</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Album_sim</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Liste_albums_pos</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Path_Possede</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Artist_A_rechercher</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Artist_Possede</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Artist_sim</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Album_A_rechercher</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Album_Possede</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Album_sim</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Liste_albums_pos</t>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Autres_albums_biblio</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>https://play.qobuz.com/album/y9763c67ocllb</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>789.15 BAS 2 (En rayon)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>789.15 BAS 2</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>/mnt/m/musiques/__Autres/Bassy Blick/Ako</t>
+          <t>Blick Bassy</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Blick Bassy</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
           <t>Bassy Blick</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="E2" t="n">
         <v>100</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1958</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1958</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>Ako</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>0</v>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Ako</t>
+        </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Ako</t>
+          <t>__Autres/Bassy Blick/Ako</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Léman - D 33151, Madiba - 789.15 BAS 2, Akö - 789.15 BAS 2</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>https://play.qobuz.com/search/%EF%BD%A5%20%EF%BD%A5%EF%BC%8D%EF%BD%A5%20%EF%BD%A5%EF%BC%8D%20%EF%BD%A5%EF%BD%A5%EF%BD%A5%20%EF%BD%A5%20%EF%BC%8D%EF%BD%A5%EF%BD%A5%20%EF%BD%A5%EF%BC%8D%EF%BD%A5%EF%BD%A5%20%EF%BD%A5%20%EF%BC%8D%20%EF%BD%A5%EF%BD%A5%20%EF%BC%8D%20%EF%BC%8D%EF%BC%8D%EF%BD%A5%20%EF%BC%8D%EF%BC%8D%EF%BC%8D</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>･ ･－･ ･－ ･･･ ･ －･･</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>･ ･－･ ･－ ･･･ ･ －･･</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
           <t>-M-</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>･－･･ ･ － ･･ － －－･ －－－</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>https://play.qobuz.com/search/%E0%B8%A7%E0%B8%87%E0%B8%94%E0%B8%B4%E0%B8%AD%E0%B8%B4%E0%B8%A1%E0%B8%9E%E0%B8%AD%E0%B8%AA%E0%B8%8B%E0%B8%B4%E0%B9%80%E0%B8%9A%E0%B8%B4%E0%B9%89%E0%B8%A5%20The%20Impossible%20%E0%B8%A3%E0%B8%A7%E0%B8%A1%E0%B8%AE%E0%B8%B4%E0%B8%95%20Vol.2</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>วงดิอิมพอสซิเบิ้ล</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>วงดิอิมพอสซิเบิ้ล</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
           <t>Haich Ber Na</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="E4" t="n">
         <v>45</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>The Impossible รวมฮิต Vol.2</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://play.qobuz.com/search/Anri%20%E6%9D%8F%E9%87%8C%20%E5%A4%8F%E7%9B%A4</t>
+          <t>https://play.qobuz.com/artist/649610</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>/mnt/m/musiques/__Autres/Anri/Timely!!</t>
+          <t>Anri</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -597,32 +601,33 @@
           <t>Anri</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Anri</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
+      <c r="E5" t="n">
         <v>100</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>杏里 夏盤</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>杏里 夏盤</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
           <t>Timely!!</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="H5" t="n">
         <v>10</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Timely!!</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Timely!!</t>
-        </is>
-      </c>
+          <t>__Autres/Anri/Timely!!</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -630,10 +635,14 @@
           <t>https://play.qobuz.com/album/bhhjotxz94fdc</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>D 43415 - Prêté (Retour prévu le : 30/05/2026)</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>/mnt/m/musiques/__Autres/Devendra Banhart/Smokey Rolls Down Thunder Canyon</t>
+          <t>Devendra Banhart</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -641,68 +650,70 @@
           <t>Devendra Banhart</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Devendra Banhart</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
+      <c r="E6" t="n">
         <v>100</v>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Cripple Crow</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Cripple Crow</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
           <t>Smokey Rolls Down Thunder Canyon</t>
         </is>
       </c>
-      <c r="I6" t="n">
+      <c r="H6" t="n">
         <v>27</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Mala - Smokey Rolls Down Thunder Canyon</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Mala - Smokey Rolls Down Thunder Canyon</t>
+          <t>__Autres/Devendra Banhart/Smokey Rolls Down Thunder Canyon</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>The black &amp; white skins vol. 1 - D 08911 V.01, Mala - D 36274 - Prêté, Flying wig - D 73150, Ma - D 65471</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>782.SOM 23 (En rayon)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>782.SOM 23</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>https://play.qobuz.com/album/tzmwwwua8jbyb</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>sombr</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>sombr</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
           <t>Colombre</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="E7" t="n">
         <v>62</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>I Barely Know Her</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -711,30 +722,35 @@
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>D3lta</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>D3lta</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
           <t>Dalida</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="E8" t="n">
         <v>55</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Kids</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Claude François, son dernier concert du 24 février 1978, Palais d'Hiver de Lyon. - Chomarat DISQ 2044, Carmen D3 - D 02288</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -743,66 +759,76 @@
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Daedr1k</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Daedr1k</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
           <t>Dxrk ダーク</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="E9" t="n">
         <v>59</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Cold Summer</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Bastien et Bastienne K. 50 : singspiel en 1 acte Lieder K. 349 et K. 351 - D 16876, Hostile : une spéciale pour les halls vol.2 - D 33067 V.02</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>https://play.qobuz.com/album/5034202018858</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>782.ARC 61 - D 67114 (En rayon - En rayon)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>782.ARC 61 - D 67114</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Arctic Monkeys</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Arctic Monkeys</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
           <t>Smoke City</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="E10" t="n">
         <v>58</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Favourite Worst Nightmare</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>AM - D 20754, Suck it and see - D 35343, Tranquility base hotel + casino - D 61055</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -811,30 +837,31 @@
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>The Cabriolets</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>The Cabriolets</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
           <t>The Cranberries</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="E11" t="n">
         <v>76</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Inside Out</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -843,138 +870,158 @@
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Elk Darling</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Elk Darling</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
           <t>David Darling</t>
         </is>
       </c>
-      <c r="F12" t="n">
+      <c r="E12" t="n">
         <v>67</v>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>The Cecil Hotel</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://play.qobuz.com/search/John%20Grant%2CSin%C3%A9ad%20O%27Connor%20Pale%20Green%20Ghosts</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t>https://play.qobuz.com/album/5414939462177</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>D 47765 (En rayon)</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>/mnt/m/musiques/__Autres/John Grant/Grey Tickles, Black Pressure</t>
+          <t>John Grant,Sinéad O'Connor</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>John Grant,Sinéad O'Connor</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
           <t>John Grant</t>
         </is>
       </c>
-      <c r="F13" t="n">
+      <c r="E13" t="n">
         <v>100</v>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Pale Green Ghosts</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Pale Green Ghosts</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
           <t>Grey Tickles, Black Pressure</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="H13" t="n">
         <v>36</v>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Boy from Michigan - Grey Tickles, Black Pressure - Queen of Denmark</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Boy from Michigan - Grey Tickles, Black Pressure - Queen of Denmark</t>
+          <t>__Autres/John Grant/Grey Tickles, Black Pressure</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Lazy dog : Deep house music mixed by Ben Watt and Jay Hannan - D 11393, The Best of Big John Patton - The organization! - D 11265</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://play.qobuz.com/search/Ghostpoet%2CPaul%20Smith%20Shedding%20Skin</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
+          <t>https://play.qobuz.com/album/5414939917257</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>D 59333 (En rayon)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ghostpoet,Paul Smith</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Ghostpoet,Paul Smith</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
           <t>Gotan Project</t>
         </is>
       </c>
-      <c r="F14" t="n">
+      <c r="E14" t="n">
         <v>64</v>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Shedding Skin</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>I grow tired but dare not fall asleep - 784.GHO 51, Some say I so I say light - D 48527, Peanut butter blues and melancholy jam - D 38552, Dark days + canapés - D 56323</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://play.qobuz.com/search/The%20Something%20Specials%2CTaylor%20Olin%20Coop</t>
+          <t>https://play.qobuz.com/album/o5bndxf773nha</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>The Something Specials,Taylor Olin</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>The Something Specials,Taylor Olin</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
           <t>nothhingspecial</t>
         </is>
       </c>
-      <c r="F15" t="n">
+      <c r="E15" t="n">
         <v>70</v>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Coop</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -983,30 +1030,31 @@
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Vlad Holiday</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Vlad Holiday</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
           <t>Hola Hola</t>
         </is>
       </c>
-      <c r="F16" t="n">
+      <c r="E16" t="n">
         <v>67</v>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Write Me off the Show</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1015,41 +1063,42 @@
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Nep</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Nep</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
           <t>Inerpol</t>
         </is>
       </c>
-      <c r="F17" t="n">
+      <c r="E17" t="n">
         <v>60</v>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Noelle</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://play.qobuz.com/search/Traf%20Quetzal</t>
+          <t>https://play.qobuz.com/artist/2591143</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>/mnt/m/musiques/__Autres/Traf/La Dibona</t>
+          <t>Traf</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1057,32 +1106,33 @@
           <t>Traf</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Traf</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
+      <c r="E18" t="n">
         <v>100</v>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Quetzal</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Quetzal</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
           <t>La Dibona</t>
         </is>
       </c>
-      <c r="I18" t="n">
+      <c r="H18" t="n">
         <v>25</v>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>John Wolfgang II - La Dibona - My Mowl</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>John Wolfgang II - La Dibona - My Mowl</t>
-        </is>
-      </c>
+          <t>__Autres/Traf/La Dibona</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1091,30 +1141,35 @@
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Renard Tortue</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Renard Tortue</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
           <t>La Tordue</t>
         </is>
       </c>
-      <c r="F19" t="n">
+      <c r="E19" t="n">
         <v>64</v>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Jamais d'accord</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Les fables de La Fontaine en chansons - D 56971</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1123,72 +1178,78 @@
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>James Supercave</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>James Supercave</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
           <t>James Spiteri</t>
         </is>
       </c>
-      <c r="F20" t="n">
+      <c r="E20" t="n">
         <v>71</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Better Strange</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://play.qobuz.com/search/Karen%20O%2CMichael%20Kiwanuka%20YO%21%20MY%20SAINT%20%28Radio%20Version%29</t>
+          <t>https://play.qobuz.com/album/u0svuxiapvfrb</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>/mnt/m/musiques/__Autres/Karen O/Crush Songs</t>
+          <t>Karen O,Michael Kiwanuka</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Karen O,Michael Kiwanuka</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
           <t>Karen O</t>
         </is>
       </c>
-      <c r="F21" t="n">
+      <c r="E21" t="n">
         <v>100</v>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>YO! MY SAINT (Radio Version)</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>YO! MY SAINT (Radio Version)</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
           <t>Crush Songs</t>
         </is>
       </c>
-      <c r="I21" t="n">
+      <c r="H21" t="n">
         <v>27</v>
       </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Crush Songs - Lux Prima - Where The Wild Things Are Motion Pic</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Crush Songs - Lux Prima - Where The Wild Things Are Motion Pic</t>
+          <t>__Autres/Karen O/Crush Songs</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Femmes celtes = Celtic women - 789.7 A 082, Crush songs - D 46851</t>
         </is>
       </c>
     </row>
@@ -1199,62 +1260,64 @@
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Disappeared Completely</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Disappeared Completely</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
           <t>Part Company</t>
         </is>
       </c>
-      <c r="F22" t="n">
+      <c r="E22" t="n">
         <v>53</v>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Not With Me</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://play.qobuz.com/search/Dirty%20Nice%20Surrenderland</t>
+          <t>https://play.qobuz.com/artist/7833010</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Dirty Nice</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Dirty Nice</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
           <t>Jane Dire</t>
         </is>
       </c>
-      <c r="F23" t="n">
+      <c r="E23" t="n">
         <v>63</v>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Surrenderland</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1263,30 +1326,31 @@
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Kanadia</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
+          <t>Nada</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>73</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>Kanadia</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Nada</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>73</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Kanadia</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1295,30 +1359,31 @@
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Kosco</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kosco</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
           <t>Coco</t>
         </is>
       </c>
-      <c r="F25" t="n">
+      <c r="E25" t="n">
         <v>67</v>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Supermoon</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1327,30 +1392,31 @@
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Pixey</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Pixey</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
           <t>Ibeyi</t>
         </is>
       </c>
-      <c r="F26" t="n">
+      <c r="E26" t="n">
         <v>60</v>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Free to Live in Colour</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="n">
-        <v>0</v>
-      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1359,30 +1425,31 @@
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>FIL BO RIVA</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>FIL BO RIVA</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
           <t>Boris Vian</t>
         </is>
       </c>
-      <c r="F27" t="n">
+      <c r="E27" t="n">
         <v>57</v>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Beautiful Sadness (Deluxe Edition)</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="n">
-        <v>0</v>
-      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1391,30 +1458,35 @@
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Gracie Abrams</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Gracie Abrams</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
           <t>Brace! Brace!</t>
         </is>
       </c>
-      <c r="F28" t="n">
+      <c r="E28" t="n">
         <v>67</v>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>The Secret of Us (Deluxe)</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="n">
-        <v>0</v>
-      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Good riddance - D 69969, The secret of us - 782.ABR 23</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1425,7 +1497,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>/mnt/m/musiques/__Autres/To Athena/The Movie</t>
+          <t>To Athena</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1433,32 +1505,33 @@
           <t>To Athena</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>To Athena</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
+      <c r="E29" t="n">
         <v>100</v>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Weird Kid</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Weird Kid</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
           <t>The Movie</t>
         </is>
       </c>
-      <c r="I29" t="n">
+      <c r="H29" t="n">
         <v>33</v>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Aquatic Ballet - Dänke - The Movie - Wältuntergang</t>
+        </is>
+      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Aquatic Ballet - Dänke - The Movie - Wältuntergang</t>
-        </is>
-      </c>
+          <t>__Autres/To Athena/The Movie</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1467,30 +1540,31 @@
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Baby Bugs</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Baby Bugs</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
           <t>BB Brunes</t>
         </is>
       </c>
-      <c r="F30" t="n">
+      <c r="E30" t="n">
         <v>67</v>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Bible Belt</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="n">
-        <v>0</v>
-      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1499,30 +1573,31 @@
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Ea Othilde</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Ea Othilde</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
           <t>White Sea</t>
         </is>
       </c>
-      <c r="F31" t="n">
+      <c r="E31" t="n">
         <v>63</v>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>I Will Not Be Like That</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="n">
-        <v>0</v>
-      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1531,30 +1606,31 @@
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Mood Bored</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Mood Bored</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
           <t>Bedroom</t>
         </is>
       </c>
-      <c r="F32" t="n">
+      <c r="E32" t="n">
         <v>59</v>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Lucky</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="n">
-        <v>0</v>
-      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1563,30 +1639,31 @@
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Blood Red Sun</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Blood Red Sun</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
           <t>Blonde Redhead</t>
         </is>
       </c>
-      <c r="F33" t="n">
+      <c r="E33" t="n">
         <v>59</v>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Pressure Lover</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="n">
-        <v>0</v>
-      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1595,30 +1672,31 @@
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Melissa Mary Ahern</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Melissa Mary Ahern</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
           <t>Melissa Auf der Maur</t>
         </is>
       </c>
-      <c r="F34" t="n">
+      <c r="E34" t="n">
         <v>79</v>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Kerosene</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="n">
-        <v>0</v>
-      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1629,7 +1707,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>/mnt/m/musiques/__Autres/Odd Beholder/Sunny Bay</t>
+          <t>Odd Beholder</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1637,32 +1715,33 @@
           <t>Odd Beholder</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Odd Beholder</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
+      <c r="E35" t="n">
         <v>100</v>
       </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Internet Famous</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Internet Famous</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
           <t>Sunny Bay</t>
         </is>
       </c>
-      <c r="I35" t="n">
+      <c r="H35" t="n">
         <v>33</v>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Drive - Feel Better - Hurt - Lighting - Remixes - Sunny Bay</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Drive - Feel Better - Hurt - Lighting - Remixes - Sunny Bay</t>
-        </is>
-      </c>
+          <t>__Autres/Odd Beholder/Sunny Bay</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1671,30 +1750,35 @@
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Esther</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Esther</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
           <t>Easter</t>
         </is>
       </c>
-      <c r="F36" t="n">
+      <c r="E36" t="n">
         <v>83</v>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Miss Congeniality</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="n">
-        <v>0</v>
-      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Esther : HWV 50 : oratorio en 6 scènes - D 34362, The Best of Esther Phillips - D 33617</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1703,30 +1787,31 @@
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>RVE</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>RVE</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
           <t>Hervé</t>
         </is>
       </c>
-      <c r="F37" t="n">
+      <c r="E37" t="n">
         <v>75</v>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="n">
-        <v>0</v>
-      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1735,30 +1820,31 @@
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Alice Costelloe</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Alice Costelloe</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
           <t>Steel Alive</t>
         </is>
       </c>
-      <c r="F38" t="n">
+      <c r="E38" t="n">
         <v>69</v>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Move On With The Year</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="n">
-        <v>0</v>
-      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1767,72 +1853,78 @@
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Alice Costelloe</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Alice Costelloe</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
           <t>Steel Alive</t>
         </is>
       </c>
-      <c r="F39" t="n">
+      <c r="E39" t="n">
         <v>69</v>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>When It's the Time</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="n">
-        <v>0</v>
-      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://play.qobuz.com/search/Laurent%20Bardainne%2CMelissa%20Weikart%20This%20Is%20Your%20Song</t>
+          <t>https://play.qobuz.com/album/e1svycay1kbko</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>/mnt/m/musiques/__Autres/Laurent Bardainne/En Amour - Adrien M &amp; Claire B (Bande originale)</t>
+          <t>Laurent Bardainne,Melissa Weikart</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Laurent Bardainne,Melissa Weikart</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
           <t>Laurent Bardainne</t>
         </is>
       </c>
-      <c r="F40" t="n">
+      <c r="E40" t="n">
         <v>100</v>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>This Is Your Song</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>This Is Your Song</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
           <t>En Amour - Adrien M &amp; Claire B (Bande originale)</t>
         </is>
       </c>
-      <c r="I40" t="n">
+      <c r="H40" t="n">
         <v>28</v>
       </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>En Amour - Adrien M &amp; Claire B (Bande originale)</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>En Amour - Adrien M &amp; Claire B (Bande originale)</t>
+          <t>__Autres/Laurent Bardainne/En Amour - Adrien M &amp; Claire B (Bande originale)</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Eden Beach Club - 781.3 BAR 8, Love is everywhere - 781.3 BAR 8 - Prêté, Hymne au soleil - 781.3 BAR 8</t>
         </is>
       </c>
     </row>
@@ -1843,66 +1935,72 @@
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Malummí</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Malummí</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
           <t>MaMaMa</t>
         </is>
       </c>
-      <c r="F41" t="n">
+      <c r="E41" t="n">
         <v>62</v>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Damaged By Their Silence</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="n">
-        <v>0</v>
-      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>https://play.qobuz.com/album/ewqnf9v3ib9am</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>782.LOW 36 (En rayon)</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>782.LOW 36</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
           <t>Elbow</t>
         </is>
       </c>
-      <c r="F42" t="n">
+      <c r="E42" t="n">
         <v>75</v>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Ones and Sixes</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="n">
-        <v>0</v>
-      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>High/low - D 49079, "Low" Symphony : symphonie n°1 - 783.GLA 24</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1911,66 +2009,72 @@
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Maudlin Strangers</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Maudlin Strangers</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
           <t>Serena Stranger</t>
         </is>
       </c>
-      <c r="F43" t="n">
+      <c r="E43" t="n">
         <v>62</v>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Silver Stain</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="n">
-        <v>0</v>
-      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>https://play.qobuz.com/album/0016861808105</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>D 34172 (En rayon)</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>D 34172</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>The Dresden Dolls</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>The Dresden Dolls</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
           <t>The Doors</t>
         </is>
       </c>
-      <c r="F44" t="n">
+      <c r="E44" t="n">
         <v>62</v>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>Yes, Virginia</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="n">
-        <v>0</v>
-      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>The Dresden Dolls - D 33324, No, Virginia... - D 24020, A is for accident - D 26475</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>